<commit_message>
London-Reise: in zwei Abrechnungen getrennt
Die Reise lief fuer CGT. Beide Fluege hat die Coldewey Holding gezahlt,
alles Uebrige Sascha privat. Daraus zwei Dokumente statt einem:

- Weiterbelastung Fluege Holding an CGT, 201,95 EUR
- Reisekosten Sascha an CGT, 267,98 EUR zuzueglich Hotel

Hinflug BA Frankfurt-London 111,97 EUR aus der Opodo-Buchung 25549979827
ergaenzt, damit sind beide Fluege belegt. Die bisherige kombinierte Datei
ist ersetzt.

Muster und die zwei offenen Steuerfragen in wissen/reisekosten.md
festgehalten: Umsatzsteuer auf die Weiterbelastung, und ob CGT die
Verpflegungspauschale steuerfrei erstatten darf.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2Vxc1sWTkdQ9c9u5jSatw
</commit_message>
<xml_diff>
--- a/templates/reisekostenabrechnung-vorlage.xlsx
+++ b/templates/reisekostenabrechnung-vorlage.xlsx
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="92">
   <si>
     <t xml:space="preserve">Reisekostenabrechnung</t>
   </si>
@@ -91,10 +91,7 @@
     <t xml:space="preserve">Inland und Ausland · Stand 2026 · Sätze siehe Blatt „Saetze 2026“</t>
   </si>
   <si>
-    <t xml:space="preserve">Firma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coldewey Holding</t>
+    <t xml:space="preserve">Abrechnung an</t>
   </si>
   <si>
     <t xml:space="preserve">Gelb = ausfüllen</t>
@@ -107,9 +104,6 @@
   </si>
   <si>
     <t xml:space="preserve">Funktion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Managing Director</t>
   </si>
   <si>
     <t xml:space="preserve">Reisezweck</t>
@@ -962,42 +956,38 @@
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>3</v>
-      </c>
+      <c r="B4" s="4"/>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
       <c r="G4" s="5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="G5" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>8</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="B6" s="4"/>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -1006,7 +996,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -1015,7 +1005,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1024,7 +1014,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -1033,7 +1023,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -1042,7 +1032,7 @@
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
@@ -1055,22 +1045,22 @@
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="D14" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="E14" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="I14" s="7" t="s">
         <v>18</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="I14" s="7" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1144,7 +1134,7 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12"/>
       <c r="B19" s="13" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C19" s="12"/>
       <c r="D19" s="12"/>
@@ -1159,7 +1149,7 @@
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -1172,16 +1162,16 @@
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1275,7 +1265,7 @@
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12"/>
       <c r="B31" s="13" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C31" s="12"/>
       <c r="D31" s="12"/>
@@ -1290,7 +1280,7 @@
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B33" s="6"/>
       <c r="C33" s="6"/>
@@ -1303,31 +1293,31 @@
     </row>
     <row r="34" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B34" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D34" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="E34" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="F34" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="E34" s="7" t="s">
+      <c r="G34" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="F34" s="7" t="s">
+      <c r="H34" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="G34" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="H34" s="7" t="s">
-        <v>33</v>
-      </c>
       <c r="I34" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1453,7 +1443,7 @@
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="12"/>
       <c r="B41" s="13" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C41" s="12"/>
       <c r="D41" s="12"/>
@@ -1468,7 +1458,7 @@
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="6"/>
@@ -1481,16 +1471,16 @@
     </row>
     <row r="44" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="I44" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1529,7 +1519,7 @@
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="12"/>
       <c r="B48" s="13" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C48" s="12"/>
       <c r="D48" s="12"/>
@@ -1544,7 +1534,7 @@
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="6"/>
@@ -1557,16 +1547,16 @@
     </row>
     <row r="51" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I51" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1616,7 +1606,7 @@
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="12"/>
       <c r="B56" s="13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C56" s="12"/>
       <c r="D56" s="12"/>
@@ -1631,7 +1621,7 @@
     </row>
     <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B58" s="6"/>
       <c r="C58" s="6"/>
@@ -1644,7 +1634,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="I59" s="18" t="n">
         <f aca="false">I19+I31+I41+I48+I56</f>
@@ -1653,20 +1643,20 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="19" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I60" s="16"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I61" s="16"/>
     </row>
     <row r="62" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="20"/>
       <c r="B62" s="21" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C62" s="20"/>
       <c r="D62" s="20"/>
@@ -1681,23 +1671,23 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="19" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E65" s="19" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B69" s="6"/>
       <c r="C69" s="6"/>
@@ -1710,10 +1700,10 @@
     </row>
     <row r="70" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="23" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B70" s="24" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C70" s="24"/>
       <c r="D70" s="24"/>
@@ -1726,7 +1716,7 @@
     <row r="71" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="23"/>
       <c r="B71" s="24" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C71" s="24"/>
       <c r="D71" s="24"/>
@@ -1739,7 +1729,7 @@
     <row r="72" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="23"/>
       <c r="B72" s="24" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C72" s="24"/>
       <c r="D72" s="24"/>
@@ -1751,10 +1741,10 @@
     </row>
     <row r="73" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="23" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B73" s="24" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C73" s="24"/>
       <c r="D73" s="24"/>
@@ -1766,10 +1756,10 @@
     </row>
     <row r="74" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="23" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B74" s="24" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C74" s="24"/>
       <c r="D74" s="24"/>
@@ -1781,10 +1771,10 @@
     </row>
     <row r="75" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="23" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B75" s="24" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C75" s="24"/>
       <c r="D75" s="24"/>
@@ -1796,10 +1786,10 @@
     </row>
     <row r="76" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="23" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B76" s="24" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C76" s="24"/>
       <c r="D76" s="24"/>
@@ -1811,10 +1801,10 @@
     </row>
     <row r="77" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="23" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B77" s="24" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C77" s="24"/>
       <c r="D77" s="24"/>
@@ -1917,43 +1907,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="E4" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="F4" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="G4" s="7" t="s">
         <v>69</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>28</v>
@@ -1968,15 +1958,15 @@
         <v>0</v>
       </c>
       <c r="G5" s="26" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C6" s="26" t="n">
         <v>66</v>
@@ -1996,10 +1986,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C7" s="26" t="n">
         <v>52</v>
@@ -2019,12 +2009,12 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B10" s="27" t="n">
         <v>0.2</v>
@@ -2032,7 +2022,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B11" s="27" t="n">
         <v>0.4</v>
@@ -2040,7 +2030,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B12" s="27" t="n">
         <v>0.4</v>
@@ -2048,12 +2038,12 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0.3</v>
@@ -2061,7 +2051,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0.2</v>
@@ -2069,7 +2059,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C17" s="28" t="n">
         <v>0.05</v>
@@ -2077,42 +2067,42 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>